<commit_message>
adicionado TRL por US
</commit_message>
<xml_diff>
--- a/reports/CV/template/Template Carga Viral.xlsx
+++ b/reports/CV/template/Template Carga Viral.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazar\weekly-reports\reports\CV\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33DC88B-C65B-4AC5-B5DF-9082D0CF3E8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6C9FCD-77A1-4686-A08A-9FFAA1E21840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="597" xr2:uid="{23642BBE-ED0C-49F7-B2BA-E2D7AA81D500}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="597" firstSheet="1" activeTab="3" xr2:uid="{23642BBE-ED0C-49F7-B2BA-E2D7AA81D500}"/>
   </bookViews>
   <sheets>
     <sheet name="Capacidade Laboratorial" sheetId="4" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Capacidade Laboratorial'!$B$2:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Tempo de Transporte'!$F$1:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TRL por US'!$F$2:$F$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TRL por US'!$F$2:$F$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -826,18 +826,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -865,6 +880,24 @@
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -877,41 +910,8 @@
     <xf numFmtId="0" fontId="10" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="10" fillId="18" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1253,38 +1253,38 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="56" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
     </row>
     <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="1:5" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="79" t="s">
+      <c r="A4" s="57" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="80" t="s">
+      <c r="B4" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="81" t="s">
+      <c r="C4" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="81" t="s">
+      <c r="D4" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="E4" s="82"/>
+      <c r="E4" s="63"/>
     </row>
     <row r="5" spans="1:5" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="56"/>
-      <c r="B5" s="57"/>
-      <c r="C5" s="58"/>
+      <c r="A5" s="58"/>
+      <c r="B5" s="60"/>
+      <c r="C5" s="62"/>
       <c r="D5" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="83" t="s">
+      <c r="E5" s="55" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1332,32 +1332,32 @@
       <c r="F2"/>
     </row>
     <row r="3" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="59"/>
-      <c r="D3" s="59"/>
-      <c r="E3" s="59"/>
-      <c r="F3" s="59"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
     </row>
     <row r="5" spans="1:15" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="60" t="s">
+      <c r="A5" s="65" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="66" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="61"/>
-      <c r="E5" s="61"/>
-      <c r="F5" s="61"/>
-      <c r="G5" s="61"/>
+      <c r="D5" s="66"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="66"/>
+      <c r="G5" s="66"/>
     </row>
     <row r="6" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="60"/>
-      <c r="B6" s="61"/>
+      <c r="A6" s="65"/>
+      <c r="B6" s="66"/>
       <c r="C6" s="16" t="s">
         <v>28</v>
       </c>
@@ -1557,10 +1557,10 @@
       <c r="O20" s="13"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="62" t="s">
+      <c r="A21" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="63">
+      <c r="B21" s="68">
         <f t="shared" ref="B21:G21" si="0">SUM(B7:B20)</f>
         <v>0</v>
       </c>
@@ -1587,8 +1587,8 @@
       <c r="O21" s="13"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="62"/>
-      <c r="B22" s="63"/>
+      <c r="A22" s="67"/>
+      <c r="B22" s="68"/>
       <c r="C22" s="15" t="e">
         <f>C21/B21</f>
         <v>#DIV/0!</v>
@@ -1730,48 +1730,48 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:26" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="67" t="s">
+      <c r="A3" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="71" t="s">
         <v>78</v>
       </c>
-      <c r="C3" s="66" t="s">
+      <c r="C3" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66" t="s">
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
-      <c r="L3" s="66" t="s">
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71" t="s">
         <v>43</v>
       </c>
-      <c r="M3" s="66"/>
-      <c r="N3" s="66"/>
-      <c r="O3" s="66" t="s">
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="66"/>
-      <c r="Q3" s="66"/>
-      <c r="R3" s="66"/>
-      <c r="S3" s="64" t="s">
+      <c r="P3" s="71"/>
+      <c r="Q3" s="71"/>
+      <c r="R3" s="71"/>
+      <c r="S3" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="66" t="s">
+      <c r="T3" s="71" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="66"/>
-      <c r="V3" s="66"/>
+      <c r="U3" s="71"/>
+      <c r="V3" s="71"/>
     </row>
     <row r="4" spans="1:26" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="67"/>
-      <c r="B4" s="66"/>
+      <c r="A4" s="72"/>
+      <c r="B4" s="71"/>
       <c r="C4" s="42" t="s">
         <v>28</v>
       </c>
@@ -1820,7 +1820,7 @@
       <c r="R4" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="S4" s="65"/>
+      <c r="S4" s="70"/>
       <c r="T4" s="42" t="s">
         <v>13</v>
       </c>
@@ -2307,30 +2307,30 @@
       <c r="A23" s="32"/>
     </row>
     <row r="24" spans="1:22" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="67" t="s">
+      <c r="A24" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="B24" s="64" t="s">
+      <c r="B24" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="66" t="s">
+      <c r="C24" s="71" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-      <c r="F24" s="66"/>
-      <c r="G24" s="66"/>
-      <c r="H24" s="66" t="s">
+      <c r="D24" s="71"/>
+      <c r="E24" s="71"/>
+      <c r="F24" s="71"/>
+      <c r="G24" s="71"/>
+      <c r="H24" s="71" t="s">
         <v>42</v>
       </c>
-      <c r="I24" s="66"/>
-      <c r="J24" s="66"/>
-      <c r="K24" s="66"/>
-      <c r="L24" s="66"/>
+      <c r="I24" s="71"/>
+      <c r="J24" s="71"/>
+      <c r="K24" s="71"/>
+      <c r="L24" s="71"/>
     </row>
     <row r="25" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="67"/>
-      <c r="B25" s="65"/>
+      <c r="A25" s="72"/>
+      <c r="B25" s="70"/>
       <c r="C25" s="42" t="s">
         <v>28</v>
       </c>
@@ -2717,7 +2717,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BBF8DF5-F4DF-45C4-BC8F-169C9A4F03E6}">
-  <dimension ref="A2:AI43"/>
+  <dimension ref="A2:AI6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" style="1" customWidth="1"/>
@@ -2758,96 +2758,96 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:35" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="79" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
     </row>
     <row r="4" spans="1:35" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="80" t="s">
         <v>68</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="81" t="s">
         <v>67</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="D4" s="71" t="s">
+      <c r="D4" s="82" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="71" t="s">
+      <c r="E4" s="82" t="s">
         <v>70</v>
       </c>
-      <c r="F4" s="71" t="s">
+      <c r="F4" s="82" t="s">
         <v>49</v>
       </c>
-      <c r="G4" s="72" t="s">
+      <c r="G4" s="73" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="72" t="s">
+      <c r="H4" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="I4" s="72" t="s">
+      <c r="I4" s="73" t="s">
         <v>64</v>
       </c>
-      <c r="J4" s="73" t="s">
+      <c r="J4" s="74" t="s">
         <v>63</v>
       </c>
-      <c r="K4" s="72" t="s">
+      <c r="K4" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="L4" s="72"/>
-      <c r="M4" s="72"/>
-      <c r="N4" s="72"/>
-      <c r="O4" s="72"/>
-      <c r="P4" s="75" t="s">
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="76" t="s">
         <v>52</v>
       </c>
-      <c r="Q4" s="76"/>
-      <c r="R4" s="76"/>
-      <c r="S4" s="76"/>
-      <c r="T4" s="77"/>
-      <c r="U4" s="75" t="s">
+      <c r="Q4" s="77"/>
+      <c r="R4" s="77"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="78"/>
+      <c r="U4" s="76" t="s">
         <v>53</v>
       </c>
-      <c r="V4" s="76"/>
-      <c r="W4" s="76"/>
-      <c r="X4" s="76"/>
-      <c r="Y4" s="77"/>
-      <c r="Z4" s="75" t="s">
+      <c r="V4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="77"/>
+      <c r="Y4" s="78"/>
+      <c r="Z4" s="76" t="s">
         <v>54</v>
       </c>
-      <c r="AA4" s="76"/>
-      <c r="AB4" s="76"/>
-      <c r="AC4" s="77"/>
-      <c r="AD4" s="75" t="s">
+      <c r="AA4" s="77"/>
+      <c r="AB4" s="77"/>
+      <c r="AC4" s="78"/>
+      <c r="AD4" s="76" t="s">
         <v>33</v>
       </c>
-      <c r="AE4" s="76"/>
-      <c r="AF4" s="76"/>
-      <c r="AG4" s="76"/>
-      <c r="AH4" s="77"/>
-      <c r="AI4" s="72" t="s">
+      <c r="AE4" s="77"/>
+      <c r="AF4" s="77"/>
+      <c r="AG4" s="77"/>
+      <c r="AH4" s="78"/>
+      <c r="AI4" s="73" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:35" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="69"/>
-      <c r="B5" s="70"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="72"/>
-      <c r="I5" s="72"/>
-      <c r="J5" s="74"/>
+      <c r="A5" s="80"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="73"/>
+      <c r="J5" s="75"/>
       <c r="K5" s="44" t="s">
         <v>28</v>
       </c>
@@ -2920,7 +2920,7 @@
       <c r="AH5" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="AI5" s="72"/>
+      <c r="AI5" s="73"/>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
@@ -2959,1385 +2959,8 @@
       <c r="AH6" s="46"/>
       <c r="AI6" s="14"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
-      <c r="U7" s="22"/>
-      <c r="V7" s="22"/>
-      <c r="W7" s="22"/>
-      <c r="X7" s="22"/>
-      <c r="Y7" s="22"/>
-      <c r="Z7" s="20"/>
-      <c r="AA7" s="20"/>
-      <c r="AB7" s="20"/>
-      <c r="AC7" s="20"/>
-      <c r="AD7" s="46"/>
-      <c r="AE7" s="46"/>
-      <c r="AF7" s="46"/>
-      <c r="AG7" s="46"/>
-      <c r="AH7" s="46"/>
-      <c r="AI7" s="14"/>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="45"/>
-      <c r="Q8" s="45"/>
-      <c r="R8" s="45"/>
-      <c r="S8" s="45"/>
-      <c r="T8" s="45"/>
-      <c r="U8" s="22"/>
-      <c r="V8" s="22"/>
-      <c r="W8" s="22"/>
-      <c r="X8" s="22"/>
-      <c r="Y8" s="22"/>
-      <c r="Z8" s="20"/>
-      <c r="AA8" s="20"/>
-      <c r="AB8" s="20"/>
-      <c r="AC8" s="20"/>
-      <c r="AD8" s="46"/>
-      <c r="AE8" s="46"/>
-      <c r="AF8" s="46"/>
-      <c r="AG8" s="46"/>
-      <c r="AH8" s="46"/>
-      <c r="AI8" s="14"/>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="45"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="22"/>
-      <c r="V9" s="22"/>
-      <c r="W9" s="22"/>
-      <c r="X9" s="22"/>
-      <c r="Y9" s="22"/>
-      <c r="Z9" s="20"/>
-      <c r="AA9" s="20"/>
-      <c r="AB9" s="20"/>
-      <c r="AC9" s="20"/>
-      <c r="AD9" s="46"/>
-      <c r="AE9" s="46"/>
-      <c r="AF9" s="46"/>
-      <c r="AG9" s="46"/>
-      <c r="AH9" s="46"/>
-      <c r="AI9" s="14"/>
-    </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="50"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="45"/>
-      <c r="Q10" s="45"/>
-      <c r="R10" s="45"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="45"/>
-      <c r="U10" s="22"/>
-      <c r="V10" s="22"/>
-      <c r="W10" s="22"/>
-      <c r="X10" s="22"/>
-      <c r="Y10" s="22"/>
-      <c r="Z10" s="20"/>
-      <c r="AA10" s="20"/>
-      <c r="AB10" s="20"/>
-      <c r="AC10" s="20"/>
-      <c r="AD10" s="46"/>
-      <c r="AE10" s="46"/>
-      <c r="AF10" s="46"/>
-      <c r="AG10" s="46"/>
-      <c r="AH10" s="46"/>
-      <c r="AI10" s="14"/>
-    </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="50"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="45"/>
-      <c r="Q11" s="45"/>
-      <c r="R11" s="45"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="45"/>
-      <c r="U11" s="22"/>
-      <c r="V11" s="22"/>
-      <c r="W11" s="22"/>
-      <c r="X11" s="22"/>
-      <c r="Y11" s="22"/>
-      <c r="Z11" s="20"/>
-      <c r="AA11" s="20"/>
-      <c r="AB11" s="20"/>
-      <c r="AC11" s="20"/>
-      <c r="AD11" s="46"/>
-      <c r="AE11" s="46"/>
-      <c r="AF11" s="46"/>
-      <c r="AG11" s="46"/>
-      <c r="AH11" s="46"/>
-      <c r="AI11" s="14"/>
-    </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="50"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="45"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="45"/>
-      <c r="S12" s="45"/>
-      <c r="T12" s="45"/>
-      <c r="U12" s="22"/>
-      <c r="V12" s="22"/>
-      <c r="W12" s="22"/>
-      <c r="X12" s="22"/>
-      <c r="Y12" s="22"/>
-      <c r="Z12" s="20"/>
-      <c r="AA12" s="20"/>
-      <c r="AB12" s="20"/>
-      <c r="AC12" s="20"/>
-      <c r="AD12" s="46"/>
-      <c r="AE12" s="46"/>
-      <c r="AF12" s="46"/>
-      <c r="AG12" s="46"/>
-      <c r="AH12" s="46"/>
-      <c r="AI12" s="14"/>
-    </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="50"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="45"/>
-      <c r="Q13" s="45"/>
-      <c r="R13" s="45"/>
-      <c r="S13" s="45"/>
-      <c r="T13" s="45"/>
-      <c r="U13" s="22"/>
-      <c r="V13" s="22"/>
-      <c r="W13" s="22"/>
-      <c r="X13" s="22"/>
-      <c r="Y13" s="22"/>
-      <c r="Z13" s="20"/>
-      <c r="AA13" s="20"/>
-      <c r="AB13" s="20"/>
-      <c r="AC13" s="20"/>
-      <c r="AD13" s="46"/>
-      <c r="AE13" s="46"/>
-      <c r="AF13" s="46"/>
-      <c r="AG13" s="46"/>
-      <c r="AH13" s="46"/>
-      <c r="AI13" s="14"/>
-    </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="50"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="45"/>
-      <c r="Q14" s="45"/>
-      <c r="R14" s="45"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="45"/>
-      <c r="U14" s="22"/>
-      <c r="V14" s="22"/>
-      <c r="W14" s="22"/>
-      <c r="X14" s="22"/>
-      <c r="Y14" s="22"/>
-      <c r="Z14" s="20"/>
-      <c r="AA14" s="20"/>
-      <c r="AB14" s="20"/>
-      <c r="AC14" s="20"/>
-      <c r="AD14" s="46"/>
-      <c r="AE14" s="46"/>
-      <c r="AF14" s="46"/>
-      <c r="AG14" s="46"/>
-      <c r="AH14" s="46"/>
-      <c r="AI14" s="14"/>
-    </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="50"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="45"/>
-      <c r="Q15" s="45"/>
-      <c r="R15" s="45"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="45"/>
-      <c r="U15" s="22"/>
-      <c r="V15" s="22"/>
-      <c r="W15" s="22"/>
-      <c r="X15" s="22"/>
-      <c r="Y15" s="22"/>
-      <c r="Z15" s="20"/>
-      <c r="AA15" s="20"/>
-      <c r="AB15" s="20"/>
-      <c r="AC15" s="20"/>
-      <c r="AD15" s="46"/>
-      <c r="AE15" s="46"/>
-      <c r="AF15" s="46"/>
-      <c r="AG15" s="46"/>
-      <c r="AH15" s="46"/>
-      <c r="AI15" s="14"/>
-    </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="50"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="45"/>
-      <c r="Q16" s="45"/>
-      <c r="R16" s="45"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="45"/>
-      <c r="U16" s="22"/>
-      <c r="V16" s="22"/>
-      <c r="W16" s="22"/>
-      <c r="X16" s="22"/>
-      <c r="Y16" s="22"/>
-      <c r="Z16" s="20"/>
-      <c r="AA16" s="20"/>
-      <c r="AB16" s="20"/>
-      <c r="AC16" s="20"/>
-      <c r="AD16" s="46"/>
-      <c r="AE16" s="46"/>
-      <c r="AF16" s="46"/>
-      <c r="AG16" s="46"/>
-      <c r="AH16" s="46"/>
-      <c r="AI16" s="14"/>
-    </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="50"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="45"/>
-      <c r="Q17" s="45"/>
-      <c r="R17" s="45"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="45"/>
-      <c r="U17" s="22"/>
-      <c r="V17" s="22"/>
-      <c r="W17" s="22"/>
-      <c r="X17" s="22"/>
-      <c r="Y17" s="22"/>
-      <c r="Z17" s="20"/>
-      <c r="AA17" s="20"/>
-      <c r="AB17" s="20"/>
-      <c r="AC17" s="20"/>
-      <c r="AD17" s="46"/>
-      <c r="AE17" s="46"/>
-      <c r="AF17" s="46"/>
-      <c r="AG17" s="46"/>
-      <c r="AH17" s="46"/>
-      <c r="AI17" s="14"/>
-    </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="45"/>
-      <c r="R18" s="45"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="45"/>
-      <c r="U18" s="22"/>
-      <c r="V18" s="22"/>
-      <c r="W18" s="22"/>
-      <c r="X18" s="22"/>
-      <c r="Y18" s="22"/>
-      <c r="Z18" s="20"/>
-      <c r="AA18" s="20"/>
-      <c r="AB18" s="20"/>
-      <c r="AC18" s="20"/>
-      <c r="AD18" s="46"/>
-      <c r="AE18" s="46"/>
-      <c r="AF18" s="46"/>
-      <c r="AG18" s="46"/>
-      <c r="AH18" s="46"/>
-      <c r="AI18" s="14"/>
-    </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="45"/>
-      <c r="Q19" s="45"/>
-      <c r="R19" s="45"/>
-      <c r="S19" s="45"/>
-      <c r="T19" s="45"/>
-      <c r="U19" s="22"/>
-      <c r="V19" s="22"/>
-      <c r="W19" s="22"/>
-      <c r="X19" s="22"/>
-      <c r="Y19" s="22"/>
-      <c r="Z19" s="20"/>
-      <c r="AA19" s="20"/>
-      <c r="AB19" s="20"/>
-      <c r="AC19" s="20"/>
-      <c r="AD19" s="46"/>
-      <c r="AE19" s="46"/>
-      <c r="AF19" s="46"/>
-      <c r="AG19" s="46"/>
-      <c r="AH19" s="46"/>
-      <c r="AI19" s="14"/>
-    </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="50"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="45"/>
-      <c r="Q20" s="45"/>
-      <c r="R20" s="45"/>
-      <c r="S20" s="45"/>
-      <c r="T20" s="45"/>
-      <c r="U20" s="22"/>
-      <c r="V20" s="22"/>
-      <c r="W20" s="22"/>
-      <c r="X20" s="22"/>
-      <c r="Y20" s="22"/>
-      <c r="Z20" s="20"/>
-      <c r="AA20" s="20"/>
-      <c r="AB20" s="20"/>
-      <c r="AC20" s="20"/>
-      <c r="AD20" s="46"/>
-      <c r="AE20" s="46"/>
-      <c r="AF20" s="46"/>
-      <c r="AG20" s="46"/>
-      <c r="AH20" s="46"/>
-      <c r="AI20" s="14"/>
-    </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="50"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="45"/>
-      <c r="Q21" s="45"/>
-      <c r="R21" s="45"/>
-      <c r="S21" s="45"/>
-      <c r="T21" s="45"/>
-      <c r="U21" s="22"/>
-      <c r="V21" s="22"/>
-      <c r="W21" s="22"/>
-      <c r="X21" s="22"/>
-      <c r="Y21" s="22"/>
-      <c r="Z21" s="20"/>
-      <c r="AA21" s="20"/>
-      <c r="AB21" s="20"/>
-      <c r="AC21" s="20"/>
-      <c r="AD21" s="46"/>
-      <c r="AE21" s="46"/>
-      <c r="AF21" s="46"/>
-      <c r="AG21" s="46"/>
-      <c r="AH21" s="46"/>
-      <c r="AI21" s="14"/>
-    </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="50"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="45"/>
-      <c r="Q22" s="45"/>
-      <c r="R22" s="45"/>
-      <c r="S22" s="45"/>
-      <c r="T22" s="45"/>
-      <c r="U22" s="22"/>
-      <c r="V22" s="22"/>
-      <c r="W22" s="22"/>
-      <c r="X22" s="22"/>
-      <c r="Y22" s="22"/>
-      <c r="Z22" s="20"/>
-      <c r="AA22" s="20"/>
-      <c r="AB22" s="20"/>
-      <c r="AC22" s="20"/>
-      <c r="AD22" s="46"/>
-      <c r="AE22" s="46"/>
-      <c r="AF22" s="46"/>
-      <c r="AG22" s="46"/>
-      <c r="AH22" s="46"/>
-      <c r="AI22" s="14"/>
-    </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="50"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="6"/>
-      <c r="P23" s="45"/>
-      <c r="Q23" s="45"/>
-      <c r="R23" s="45"/>
-      <c r="S23" s="45"/>
-      <c r="T23" s="45"/>
-      <c r="U23" s="22"/>
-      <c r="V23" s="22"/>
-      <c r="W23" s="22"/>
-      <c r="X23" s="22"/>
-      <c r="Y23" s="22"/>
-      <c r="Z23" s="20"/>
-      <c r="AA23" s="20"/>
-      <c r="AB23" s="20"/>
-      <c r="AC23" s="20"/>
-      <c r="AD23" s="46"/>
-      <c r="AE23" s="46"/>
-      <c r="AF23" s="46"/>
-      <c r="AG23" s="46"/>
-      <c r="AH23" s="46"/>
-      <c r="AI23" s="14"/>
-    </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="50"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="6"/>
-      <c r="P24" s="45"/>
-      <c r="Q24" s="45"/>
-      <c r="R24" s="45"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="45"/>
-      <c r="U24" s="22"/>
-      <c r="V24" s="22"/>
-      <c r="W24" s="22"/>
-      <c r="X24" s="22"/>
-      <c r="Y24" s="22"/>
-      <c r="Z24" s="20"/>
-      <c r="AA24" s="20"/>
-      <c r="AB24" s="20"/>
-      <c r="AC24" s="20"/>
-      <c r="AD24" s="46"/>
-      <c r="AE24" s="46"/>
-      <c r="AF24" s="46"/>
-      <c r="AG24" s="46"/>
-      <c r="AH24" s="46"/>
-      <c r="AI24" s="14"/>
-    </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="50"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="45"/>
-      <c r="Q25" s="45"/>
-      <c r="R25" s="45"/>
-      <c r="S25" s="45"/>
-      <c r="T25" s="45"/>
-      <c r="U25" s="22"/>
-      <c r="V25" s="22"/>
-      <c r="W25" s="22"/>
-      <c r="X25" s="22"/>
-      <c r="Y25" s="22"/>
-      <c r="Z25" s="20"/>
-      <c r="AA25" s="20"/>
-      <c r="AB25" s="20"/>
-      <c r="AC25" s="20"/>
-      <c r="AD25" s="46"/>
-      <c r="AE25" s="46"/>
-      <c r="AF25" s="46"/>
-      <c r="AG25" s="46"/>
-      <c r="AH25" s="46"/>
-      <c r="AI25" s="14"/>
-    </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="50"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="45"/>
-      <c r="Q26" s="45"/>
-      <c r="R26" s="45"/>
-      <c r="S26" s="45"/>
-      <c r="T26" s="45"/>
-      <c r="U26" s="22"/>
-      <c r="V26" s="22"/>
-      <c r="W26" s="22"/>
-      <c r="X26" s="22"/>
-      <c r="Y26" s="22"/>
-      <c r="Z26" s="20"/>
-      <c r="AA26" s="20"/>
-      <c r="AB26" s="20"/>
-      <c r="AC26" s="20"/>
-      <c r="AD26" s="46"/>
-      <c r="AE26" s="46"/>
-      <c r="AF26" s="46"/>
-      <c r="AG26" s="46"/>
-      <c r="AH26" s="46"/>
-      <c r="AI26" s="14"/>
-    </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="50"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
-      <c r="M27" s="6"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="6"/>
-      <c r="P27" s="45"/>
-      <c r="Q27" s="45"/>
-      <c r="R27" s="45"/>
-      <c r="S27" s="45"/>
-      <c r="T27" s="45"/>
-      <c r="U27" s="22"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="22"/>
-      <c r="X27" s="22"/>
-      <c r="Y27" s="22"/>
-      <c r="Z27" s="20"/>
-      <c r="AA27" s="20"/>
-      <c r="AB27" s="20"/>
-      <c r="AC27" s="20"/>
-      <c r="AD27" s="46"/>
-      <c r="AE27" s="46"/>
-      <c r="AF27" s="46"/>
-      <c r="AG27" s="46"/>
-      <c r="AH27" s="46"/>
-      <c r="AI27" s="14"/>
-    </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="34"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="45"/>
-      <c r="Q28" s="45"/>
-      <c r="R28" s="45"/>
-      <c r="S28" s="45"/>
-      <c r="T28" s="45"/>
-      <c r="U28" s="22"/>
-      <c r="V28" s="22"/>
-      <c r="W28" s="22"/>
-      <c r="X28" s="22"/>
-      <c r="Y28" s="22"/>
-      <c r="Z28" s="20"/>
-      <c r="AA28" s="20"/>
-      <c r="AB28" s="20"/>
-      <c r="AC28" s="20"/>
-      <c r="AD28" s="46"/>
-      <c r="AE28" s="46"/>
-      <c r="AF28" s="46"/>
-      <c r="AG28" s="46"/>
-      <c r="AH28" s="46"/>
-      <c r="AI28" s="14"/>
-    </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="50"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="45"/>
-      <c r="Q29" s="45"/>
-      <c r="R29" s="45"/>
-      <c r="S29" s="45"/>
-      <c r="T29" s="45"/>
-      <c r="U29" s="22"/>
-      <c r="V29" s="22"/>
-      <c r="W29" s="22"/>
-      <c r="X29" s="22"/>
-      <c r="Y29" s="22"/>
-      <c r="Z29" s="20"/>
-      <c r="AA29" s="20"/>
-      <c r="AB29" s="20"/>
-      <c r="AC29" s="20"/>
-      <c r="AD29" s="46"/>
-      <c r="AE29" s="46"/>
-      <c r="AF29" s="46"/>
-      <c r="AG29" s="46"/>
-      <c r="AH29" s="46"/>
-      <c r="AI29" s="14"/>
-    </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="50"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="45"/>
-      <c r="Q30" s="45"/>
-      <c r="R30" s="45"/>
-      <c r="S30" s="45"/>
-      <c r="T30" s="45"/>
-      <c r="U30" s="22"/>
-      <c r="V30" s="22"/>
-      <c r="W30" s="22"/>
-      <c r="X30" s="22"/>
-      <c r="Y30" s="22"/>
-      <c r="Z30" s="20"/>
-      <c r="AA30" s="20"/>
-      <c r="AB30" s="20"/>
-      <c r="AC30" s="20"/>
-      <c r="AD30" s="46"/>
-      <c r="AE30" s="46"/>
-      <c r="AF30" s="46"/>
-      <c r="AG30" s="46"/>
-      <c r="AH30" s="46"/>
-      <c r="AI30" s="14"/>
-    </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="50"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="45"/>
-      <c r="Q31" s="45"/>
-      <c r="R31" s="45"/>
-      <c r="S31" s="45"/>
-      <c r="T31" s="45"/>
-      <c r="U31" s="22"/>
-      <c r="V31" s="22"/>
-      <c r="W31" s="22"/>
-      <c r="X31" s="22"/>
-      <c r="Y31" s="22"/>
-      <c r="Z31" s="20"/>
-      <c r="AA31" s="20"/>
-      <c r="AB31" s="20"/>
-      <c r="AC31" s="20"/>
-      <c r="AD31" s="46"/>
-      <c r="AE31" s="46"/>
-      <c r="AF31" s="46"/>
-      <c r="AG31" s="46"/>
-      <c r="AH31" s="46"/>
-      <c r="AI31" s="14"/>
-    </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A32" s="3"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="50"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="45"/>
-      <c r="Q32" s="45"/>
-      <c r="R32" s="45"/>
-      <c r="S32" s="45"/>
-      <c r="T32" s="45"/>
-      <c r="U32" s="22"/>
-      <c r="V32" s="22"/>
-      <c r="W32" s="22"/>
-      <c r="X32" s="22"/>
-      <c r="Y32" s="22"/>
-      <c r="Z32" s="20"/>
-      <c r="AA32" s="20"/>
-      <c r="AB32" s="20"/>
-      <c r="AC32" s="20"/>
-      <c r="AD32" s="46"/>
-      <c r="AE32" s="46"/>
-      <c r="AF32" s="46"/>
-      <c r="AG32" s="46"/>
-      <c r="AH32" s="46"/>
-      <c r="AI32" s="14"/>
-    </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="50"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6"/>
-      <c r="P33" s="45"/>
-      <c r="Q33" s="45"/>
-      <c r="R33" s="45"/>
-      <c r="S33" s="45"/>
-      <c r="T33" s="45"/>
-      <c r="U33" s="22"/>
-      <c r="V33" s="22"/>
-      <c r="W33" s="22"/>
-      <c r="X33" s="22"/>
-      <c r="Y33" s="22"/>
-      <c r="Z33" s="20"/>
-      <c r="AA33" s="20"/>
-      <c r="AB33" s="20"/>
-      <c r="AC33" s="20"/>
-      <c r="AD33" s="46"/>
-      <c r="AE33" s="46"/>
-      <c r="AF33" s="46"/>
-      <c r="AG33" s="46"/>
-      <c r="AH33" s="46"/>
-      <c r="AI33" s="14"/>
-    </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A34" s="3"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-      <c r="I34" s="34"/>
-      <c r="J34" s="50"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="6"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="6"/>
-      <c r="P34" s="45"/>
-      <c r="Q34" s="45"/>
-      <c r="R34" s="45"/>
-      <c r="S34" s="45"/>
-      <c r="T34" s="45"/>
-      <c r="U34" s="22"/>
-      <c r="V34" s="22"/>
-      <c r="W34" s="22"/>
-      <c r="X34" s="22"/>
-      <c r="Y34" s="22"/>
-      <c r="Z34" s="20"/>
-      <c r="AA34" s="20"/>
-      <c r="AB34" s="20"/>
-      <c r="AC34" s="20"/>
-      <c r="AD34" s="46"/>
-      <c r="AE34" s="46"/>
-      <c r="AF34" s="46"/>
-      <c r="AG34" s="46"/>
-      <c r="AH34" s="46"/>
-      <c r="AI34" s="14"/>
-    </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="50"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-      <c r="N35" s="6"/>
-      <c r="O35" s="6"/>
-      <c r="P35" s="45"/>
-      <c r="Q35" s="45"/>
-      <c r="R35" s="45"/>
-      <c r="S35" s="45"/>
-      <c r="T35" s="45"/>
-      <c r="U35" s="22"/>
-      <c r="V35" s="22"/>
-      <c r="W35" s="22"/>
-      <c r="X35" s="22"/>
-      <c r="Y35" s="22"/>
-      <c r="Z35" s="20"/>
-      <c r="AA35" s="20"/>
-      <c r="AB35" s="20"/>
-      <c r="AC35" s="20"/>
-      <c r="AD35" s="46"/>
-      <c r="AE35" s="46"/>
-      <c r="AF35" s="46"/>
-      <c r="AG35" s="46"/>
-      <c r="AH35" s="46"/>
-      <c r="AI35" s="14"/>
-    </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A36" s="3"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-      <c r="I36" s="34"/>
-      <c r="J36" s="50"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="45"/>
-      <c r="Q36" s="45"/>
-      <c r="R36" s="45"/>
-      <c r="S36" s="45"/>
-      <c r="T36" s="45"/>
-      <c r="U36" s="22"/>
-      <c r="V36" s="22"/>
-      <c r="W36" s="22"/>
-      <c r="X36" s="22"/>
-      <c r="Y36" s="22"/>
-      <c r="Z36" s="20"/>
-      <c r="AA36" s="20"/>
-      <c r="AB36" s="20"/>
-      <c r="AC36" s="20"/>
-      <c r="AD36" s="46"/>
-      <c r="AE36" s="46"/>
-      <c r="AF36" s="46"/>
-      <c r="AG36" s="46"/>
-      <c r="AH36" s="46"/>
-      <c r="AI36" s="14"/>
-    </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A37" s="3"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-      <c r="I37" s="34"/>
-      <c r="J37" s="50"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="45"/>
-      <c r="Q37" s="45"/>
-      <c r="R37" s="45"/>
-      <c r="S37" s="45"/>
-      <c r="T37" s="45"/>
-      <c r="U37" s="22"/>
-      <c r="V37" s="22"/>
-      <c r="W37" s="22"/>
-      <c r="X37" s="22"/>
-      <c r="Y37" s="22"/>
-      <c r="Z37" s="20"/>
-      <c r="AA37" s="20"/>
-      <c r="AB37" s="20"/>
-      <c r="AC37" s="20"/>
-      <c r="AD37" s="46"/>
-      <c r="AE37" s="46"/>
-      <c r="AF37" s="46"/>
-      <c r="AG37" s="46"/>
-      <c r="AH37" s="46"/>
-      <c r="AI37" s="14"/>
-    </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A38" s="3"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-      <c r="I38" s="34"/>
-      <c r="J38" s="50"/>
-      <c r="K38" s="6"/>
-      <c r="L38" s="6"/>
-      <c r="M38" s="6"/>
-      <c r="N38" s="6"/>
-      <c r="O38" s="6"/>
-      <c r="P38" s="45"/>
-      <c r="Q38" s="45"/>
-      <c r="R38" s="45"/>
-      <c r="S38" s="45"/>
-      <c r="T38" s="45"/>
-      <c r="U38" s="22"/>
-      <c r="V38" s="22"/>
-      <c r="W38" s="22"/>
-      <c r="X38" s="22"/>
-      <c r="Y38" s="22"/>
-      <c r="Z38" s="20"/>
-      <c r="AA38" s="20"/>
-      <c r="AB38" s="20"/>
-      <c r="AC38" s="20"/>
-      <c r="AD38" s="46"/>
-      <c r="AE38" s="46"/>
-      <c r="AF38" s="46"/>
-      <c r="AG38" s="46"/>
-      <c r="AH38" s="46"/>
-      <c r="AI38" s="14"/>
-    </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A39" s="3"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
-      <c r="I39" s="34"/>
-      <c r="J39" s="50"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-      <c r="N39" s="6"/>
-      <c r="O39" s="6"/>
-      <c r="P39" s="45"/>
-      <c r="Q39" s="45"/>
-      <c r="R39" s="45"/>
-      <c r="S39" s="45"/>
-      <c r="T39" s="45"/>
-      <c r="U39" s="22"/>
-      <c r="V39" s="22"/>
-      <c r="W39" s="22"/>
-      <c r="X39" s="22"/>
-      <c r="Y39" s="22"/>
-      <c r="Z39" s="20"/>
-      <c r="AA39" s="20"/>
-      <c r="AB39" s="20"/>
-      <c r="AC39" s="20"/>
-      <c r="AD39" s="46"/>
-      <c r="AE39" s="46"/>
-      <c r="AF39" s="46"/>
-      <c r="AG39" s="46"/>
-      <c r="AH39" s="46"/>
-      <c r="AI39" s="14"/>
-    </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A40" s="3"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="3"/>
-      <c r="H40" s="3"/>
-      <c r="I40" s="34"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="6"/>
-      <c r="M40" s="6"/>
-      <c r="N40" s="6"/>
-      <c r="O40" s="6"/>
-      <c r="P40" s="45"/>
-      <c r="Q40" s="45"/>
-      <c r="R40" s="45"/>
-      <c r="S40" s="45"/>
-      <c r="T40" s="45"/>
-      <c r="U40" s="22"/>
-      <c r="V40" s="22"/>
-      <c r="W40" s="22"/>
-      <c r="X40" s="22"/>
-      <c r="Y40" s="22"/>
-      <c r="Z40" s="20"/>
-      <c r="AA40" s="20"/>
-      <c r="AB40" s="20"/>
-      <c r="AC40" s="20"/>
-      <c r="AD40" s="46"/>
-      <c r="AE40" s="46"/>
-      <c r="AF40" s="46"/>
-      <c r="AG40" s="46"/>
-      <c r="AH40" s="46"/>
-      <c r="AI40" s="14"/>
-    </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A41" s="3"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="34"/>
-      <c r="J41" s="50"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
-      <c r="N41" s="6"/>
-      <c r="O41" s="6"/>
-      <c r="P41" s="45"/>
-      <c r="Q41" s="45"/>
-      <c r="R41" s="45"/>
-      <c r="S41" s="45"/>
-      <c r="T41" s="45"/>
-      <c r="U41" s="22"/>
-      <c r="V41" s="22"/>
-      <c r="W41" s="22"/>
-      <c r="X41" s="22"/>
-      <c r="Y41" s="22"/>
-      <c r="Z41" s="20"/>
-      <c r="AA41" s="20"/>
-      <c r="AB41" s="20"/>
-      <c r="AC41" s="20"/>
-      <c r="AD41" s="46"/>
-      <c r="AE41" s="46"/>
-      <c r="AF41" s="46"/>
-      <c r="AG41" s="46"/>
-      <c r="AH41" s="46"/>
-      <c r="AI41" s="14"/>
-    </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A42" s="3"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="34"/>
-      <c r="J42" s="50"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="45"/>
-      <c r="Q42" s="45"/>
-      <c r="R42" s="45"/>
-      <c r="S42" s="45"/>
-      <c r="T42" s="45"/>
-      <c r="U42" s="22"/>
-      <c r="V42" s="22"/>
-      <c r="W42" s="22"/>
-      <c r="X42" s="22"/>
-      <c r="Y42" s="22"/>
-      <c r="Z42" s="20"/>
-      <c r="AA42" s="20"/>
-      <c r="AB42" s="20"/>
-      <c r="AC42" s="20"/>
-      <c r="AD42" s="46"/>
-      <c r="AE42" s="46"/>
-      <c r="AF42" s="46"/>
-      <c r="AG42" s="46"/>
-      <c r="AH42" s="46"/>
-      <c r="AI42" s="14"/>
-    </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A43" s="3"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="3"/>
-      <c r="H43" s="3"/>
-      <c r="I43" s="34"/>
-      <c r="J43" s="50"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
-      <c r="O43" s="6"/>
-      <c r="P43" s="45"/>
-      <c r="Q43" s="45"/>
-      <c r="R43" s="45"/>
-      <c r="S43" s="45"/>
-      <c r="T43" s="45"/>
-      <c r="U43" s="22"/>
-      <c r="V43" s="22"/>
-      <c r="W43" s="22"/>
-      <c r="X43" s="22"/>
-      <c r="Y43" s="22"/>
-      <c r="Z43" s="20"/>
-      <c r="AA43" s="20"/>
-      <c r="AB43" s="20"/>
-      <c r="AC43" s="20"/>
-      <c r="AD43" s="46"/>
-      <c r="AE43" s="46"/>
-      <c r="AF43" s="46"/>
-      <c r="AG43" s="46"/>
-      <c r="AH43" s="46"/>
-      <c r="AI43" s="14"/>
-    </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="AI4:AI5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="K4:O4"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="U4:Y4"/>
-    <mergeCell ref="Z4:AC4"/>
-    <mergeCell ref="AD4:AH4"/>
-    <mergeCell ref="P4:T4"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="A4:A5"/>
     <mergeCell ref="B4:B5"/>
@@ -4347,6 +2970,14 @@
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="G4:G5"/>
     <mergeCell ref="H4:H5"/>
+    <mergeCell ref="AI4:AI5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="K4:O4"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="U4:Y4"/>
+    <mergeCell ref="Z4:AC4"/>
+    <mergeCell ref="AD4:AH4"/>
+    <mergeCell ref="P4:T4"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4422,15 +3053,15 @@
       <c r="AE1" s="4"/>
     </row>
     <row r="2" spans="1:34" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="79" t="s">
         <v>82</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
       <c r="I2" s="49"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -4482,79 +3113,79 @@
       <c r="AE3" s="4"/>
     </row>
     <row r="4" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="69" t="s">
+      <c r="A4" s="80" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="78" t="s">
+      <c r="B4" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="82" t="s">
         <v>46</v>
       </c>
-      <c r="D4" s="71" t="s">
+      <c r="D4" s="82" t="s">
         <v>47</v>
       </c>
-      <c r="E4" s="71" t="s">
+      <c r="E4" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="F4" s="71" t="s">
+      <c r="F4" s="82" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="72" t="s">
+      <c r="G4" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="H4" s="72" t="s">
+      <c r="H4" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="74" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="58" t="s">
+      <c r="J4" s="62" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="58"/>
-      <c r="L4" s="58"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="58" t="s">
+      <c r="K4" s="62"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="P4" s="58"/>
-      <c r="Q4" s="58"/>
-      <c r="R4" s="58"/>
-      <c r="S4" s="58"/>
-      <c r="T4" s="58" t="s">
+      <c r="P4" s="62"/>
+      <c r="Q4" s="62"/>
+      <c r="R4" s="62"/>
+      <c r="S4" s="62"/>
+      <c r="T4" s="62" t="s">
         <v>59</v>
       </c>
-      <c r="U4" s="58"/>
-      <c r="V4" s="58"/>
-      <c r="W4" s="58"/>
-      <c r="X4" s="58"/>
-      <c r="Y4" s="58" t="s">
+      <c r="U4" s="62"/>
+      <c r="V4" s="62"/>
+      <c r="W4" s="62"/>
+      <c r="X4" s="62"/>
+      <c r="Y4" s="62" t="s">
         <v>60</v>
       </c>
-      <c r="Z4" s="58"/>
-      <c r="AA4" s="58"/>
-      <c r="AB4" s="58"/>
-      <c r="AC4" s="58"/>
-      <c r="AD4" s="58" t="s">
+      <c r="Z4" s="62"/>
+      <c r="AA4" s="62"/>
+      <c r="AB4" s="62"/>
+      <c r="AC4" s="62"/>
+      <c r="AD4" s="62" t="s">
         <v>61</v>
       </c>
-      <c r="AE4" s="58"/>
-      <c r="AF4" s="58"/>
-      <c r="AG4" s="58"/>
-      <c r="AH4" s="58"/>
+      <c r="AE4" s="62"/>
+      <c r="AF4" s="62"/>
+      <c r="AG4" s="62"/>
+      <c r="AH4" s="62"/>
     </row>
     <row r="5" spans="1:34" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="69"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
-      <c r="F5" s="71"/>
-      <c r="G5" s="72"/>
-      <c r="H5" s="72"/>
-      <c r="I5" s="74"/>
+      <c r="A5" s="80"/>
+      <c r="B5" s="83"/>
+      <c r="C5" s="82"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="75"/>
       <c r="J5" s="47" t="s">
         <v>28</v>
       </c>

</xml_diff>

<commit_message>
Adicionado Tempo de Transporte
</commit_message>
<xml_diff>
--- a/reports/CV/template/Template Carga Viral.xlsx
+++ b/reports/CV/template/Template Carga Viral.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lazar\weekly-reports\reports\CV\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6C9FCD-77A1-4686-A08A-9FFAA1E21840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E3621C-278C-4FB6-89AE-242C8345DD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="597" firstSheet="1" activeTab="3" xr2:uid="{23642BBE-ED0C-49F7-B2BA-E2D7AA81D500}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="597" xr2:uid="{23642BBE-ED0C-49F7-B2BA-E2D7AA81D500}"/>
   </bookViews>
   <sheets>
     <sheet name="Capacidade Laboratorial" sheetId="4" r:id="rId1"/>
@@ -2720,7 +2720,7 @@
   <dimension ref="A2:AI6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" style="43" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" style="24" customWidth="1"/>
     <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -2923,7 +2923,7 @@
       <c r="AI5" s="73"/>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -2990,7 +2990,7 @@
   <dimension ref="A1:AH6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" style="43" customWidth="1"/>
     <col min="2" max="2" width="16.109375" customWidth="1"/>
     <col min="3" max="3" width="17.109375" customWidth="1"/>
     <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
@@ -3263,7 +3263,7 @@
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
+      <c r="A6" s="34"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>

</xml_diff>